<commit_message>
got general program running to work
</commit_message>
<xml_diff>
--- a/VK_automation.xlsx
+++ b/VK_automation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER1\PycharmProjects\keyenceAHK\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED96D42E-7CD6-4802-8AA4-291C6A093228}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F2F66F-DD12-4B69-980A-A2E87C2AE903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="870" yWindow="405" windowWidth="17805" windowHeight="14220" xr2:uid="{0497DB16-1CCC-40D6-B601-ECD47C888558}"/>
+    <workbookView xWindow="5760" yWindow="2550" windowWidth="21390" windowHeight="10365" xr2:uid="{0497DB16-1CCC-40D6-B601-ECD47C888558}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="42">
   <si>
     <t>WindowsForms10.Window.8.app.0.2f5a4f0_r9_ad193</t>
   </si>
@@ -59,9 +59,6 @@
     <t>WindowsForms10.BUTTON.app.0.2f5a4f0_r9_ad129</t>
   </si>
   <si>
-    <t>name</t>
-  </si>
-  <si>
     <t>ClassNN</t>
   </si>
   <si>
@@ -107,9 +104,6 @@
     <t>enter_teaching_file_path</t>
   </si>
   <si>
-    <t>C:\Users\USER1\Documents\Jake\AL_9x9\gantry_procedure.vkt</t>
-  </si>
-  <si>
     <t>Button1</t>
   </si>
   <si>
@@ -122,9 +116,6 @@
     <t>Send</t>
   </si>
   <si>
-    <t>text ="Move to the 1 measurement point. Check that there is no danger of a lens collision."</t>
-  </si>
-  <si>
     <t>lens_danger_button</t>
   </si>
   <si>
@@ -146,10 +137,34 @@
     <t>C:\Users\USER1\Documents\kyle\AHK</t>
   </si>
   <si>
-    <t>var lens_danger_window</t>
-  </si>
-  <si>
     <t>var save_file_name</t>
+  </si>
+  <si>
+    <t>start_ok</t>
+  </si>
+  <si>
+    <t>WindowsForms10.BUTTON.app.0.2f5a4f0_r9_ad14</t>
+  </si>
+  <si>
+    <t>over_saturate_ok</t>
+  </si>
+  <si>
+    <t>auto_focus_ok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autofocus failed. The following locations were not </t>
+  </si>
+  <si>
+    <t>"C:\Users\USER1\Documents\Jake\AL_9x9\gantry_procedure_dummy.vkt"</t>
+  </si>
+  <si>
+    <t>text lens_danger_window</t>
+  </si>
+  <si>
+    <t>Check that there is no danger of a lens</t>
+  </si>
+  <si>
+    <t>key</t>
   </si>
 </sst>
 </file>
@@ -521,14 +536,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F659CD83-B42B-4A28-A51B-5F0CEEA4A19F}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.7109375" customWidth="1"/>
     <col min="2" max="2" width="49.42578125" customWidth="1"/>
     <col min="3" max="3" width="12.28515625" customWidth="1"/>
     <col min="4" max="4" width="11.85546875" customWidth="1"/>
-    <col min="5" max="5" width="25.7109375" customWidth="1"/>
+    <col min="5" max="5" width="57.85546875" customWidth="1"/>
     <col min="6" max="6" width="22.7109375" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" customWidth="1"/>
     <col min="8" max="8" width="27.140625" customWidth="1"/>
@@ -536,28 +551,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" t="s">
         <v>8</v>
-      </c>
-      <c r="E1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -568,16 +583,16 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -588,13 +603,13 @@
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -605,13 +620,13 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
@@ -619,22 +634,22 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
@@ -642,16 +657,19 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
@@ -659,45 +677,45 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F7" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G8" t="b">
         <v>1</v>
@@ -705,22 +723,73 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" t="s">
         <v>32</v>
       </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" t="s">
-        <v>36</v>
+      <c r="F9" t="s">
+        <v>27</v>
       </c>
       <c r="G9" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>